<commit_message>
actualizo un poco el excel
</commit_message>
<xml_diff>
--- a/resultados/doe_3factores_2niveles_r3_20260306_013644.xlsx
+++ b/resultados/doe_3factores_2niveles_r3_20260306_013644.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivija\Desktop\Simulacion Terminal La Plata\Simulacion\resultados\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://frlputneduar-my.sharepoint.com/personal/belizalde_alu_frlp_utn_edu_ar/Documents/Facultad/4to Año/Simulacion/Trabajo Integrador/Simulacion/resultados/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7D1B196-D741-4B42-82F5-1F87F9540C16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{C7D1B196-D741-4B42-82F5-1F87F9540C16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{19A8469C-C398-4FCE-9D1E-AD6148F0AAEE}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ANOVA" sheetId="2" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="37">
   <si>
     <t>corrida</t>
   </si>
@@ -145,27 +145,6 @@
   </si>
   <si>
     <t>Superior 95,0%</t>
-  </si>
-  <si>
-    <t>Variable X 4</t>
-  </si>
-  <si>
-    <t>Variable X 5</t>
-  </si>
-  <si>
-    <t>Variable X 6</t>
-  </si>
-  <si>
-    <t>Variable X 7</t>
-  </si>
-  <si>
-    <t>Variable X 1(A)</t>
-  </si>
-  <si>
-    <t>Variable X 2(S)</t>
-  </si>
-  <si>
-    <t>Variable X 3(R)</t>
   </si>
 </sst>
 </file>
@@ -208,7 +187,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -251,17 +230,6 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -271,17 +239,17 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -585,397 +553,395 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD9BFBE4-8636-4659-A232-8E71DCCF3BE3}">
   <dimension ref="A1:I24"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="32.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="32.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
+    <row r="2" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="5"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="B3" s="4"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4">
         <v>0.80659736716918562</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5">
         <v>0.65059931272426197</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6">
         <v>0.49773651204112657</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7">
         <v>258.94161925813728</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="3" t="s">
+    <row r="8" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="3">
+      <c r="B8" s="2">
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="4"/>
-      <c r="B11" s="4" t="s">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A11" s="3"/>
+      <c r="B11" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="F11" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
         <v>21</v>
       </c>
-      <c r="B12" s="2">
+      <c r="B12">
         <v>7</v>
       </c>
-      <c r="C12" s="2">
+      <c r="C12">
         <v>1997623.0789787336</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12">
         <v>285374.72556839051</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12">
         <v>4.2560996515618568</v>
       </c>
-      <c r="F12" s="2">
+      <c r="F12">
         <v>7.8219721074878259E-3</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
         <v>22</v>
       </c>
-      <c r="B13" s="2">
+      <c r="B13">
         <v>16</v>
       </c>
-      <c r="C13" s="2">
+      <c r="C13">
         <v>1072812.194944418</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13">
         <v>67050.762184026127</v>
       </c>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-    </row>
-    <row r="14" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="3" t="s">
+    </row>
+    <row r="14" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="3">
+      <c r="B14" s="2">
         <v>23</v>
       </c>
-      <c r="C14" s="3">
+      <c r="C14" s="2">
         <v>3070435.2739231517</v>
       </c>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-    </row>
-    <row r="15" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="4"/>
-      <c r="B16" s="4" t="s">
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+    </row>
+    <row r="15" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A16" s="3"/>
+      <c r="B16" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="F16" s="4" t="s">
+      <c r="F16" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="G16" s="4" t="s">
+      <c r="G16" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="H16" s="4" t="s">
+      <c r="H16" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="I16" s="4" t="s">
+      <c r="I16" s="3" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
         <v>24</v>
       </c>
-      <c r="B17" s="2">
+      <c r="B17">
         <v>1167.5599599480111</v>
       </c>
-      <c r="C17" s="2">
+      <c r="C17">
         <v>52.856236696039531</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D17">
         <v>22.089350905973511</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17">
         <v>2.0570743919978214E-13</v>
       </c>
-      <c r="F17" s="2">
+      <c r="F17">
         <v>1055.5097436791839</v>
       </c>
-      <c r="G17" s="2">
+      <c r="G17">
         <v>1279.6101762168382</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17">
         <v>1055.5097436791839</v>
       </c>
-      <c r="I17" s="2">
+      <c r="I17">
         <v>1279.6101762168382</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B18" s="2">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>5</v>
+      </c>
+      <c r="B18">
         <v>-221.05699946587029</v>
       </c>
-      <c r="C18" s="2">
+      <c r="C18">
         <v>52.856236696039531</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D18">
         <v>-4.1822311478038667</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18">
         <v>7.0418585302546815E-4</v>
       </c>
-      <c r="F18" s="2">
+      <c r="F18">
         <v>-333.10721573469743</v>
       </c>
-      <c r="G18" s="2">
+      <c r="G18">
         <v>-109.00678319704313</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18">
         <v>-333.10721573469743</v>
       </c>
-      <c r="I18" s="2">
+      <c r="I18">
         <v>-109.00678319704313</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="B19" s="2">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>6</v>
+      </c>
+      <c r="B19">
         <v>30.311398155756926</v>
       </c>
-      <c r="C19" s="2">
+      <c r="C19">
         <v>52.856236696039531</v>
       </c>
-      <c r="D19" s="2">
+      <c r="D19">
         <v>0.57346871533947352</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19">
         <v>0.57430021394171304</v>
       </c>
-      <c r="F19" s="2">
+      <c r="F19">
         <v>-81.738818113070238</v>
       </c>
-      <c r="G19" s="2">
+      <c r="G19">
         <v>142.36161442458408</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19">
         <v>-81.738818113070238</v>
       </c>
-      <c r="I19" s="2">
+      <c r="I19">
         <v>142.36161442458408</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="B20" s="2">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>7</v>
+      </c>
+      <c r="B20">
         <v>126.00339748044119</v>
       </c>
-      <c r="C20" s="2">
+      <c r="C20">
         <v>52.856236696039531</v>
       </c>
-      <c r="D20" s="2">
+      <c r="D20">
         <v>2.3838889288514653</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20">
         <v>2.9860683388170609E-2</v>
       </c>
-      <c r="F20" s="2">
+      <c r="F20">
         <v>13.953181211614037</v>
       </c>
-      <c r="G20" s="2">
+      <c r="G20">
         <v>238.05361374926835</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20">
         <v>13.953181211614037</v>
       </c>
-      <c r="I20" s="2">
+      <c r="I20">
         <v>238.05361374926835</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B21" s="2">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>9</v>
+      </c>
+      <c r="B21">
         <v>8.8641173598824476</v>
       </c>
-      <c r="C21" s="2">
+      <c r="C21">
         <v>52.856236696039524</v>
       </c>
-      <c r="D21" s="2">
+      <c r="D21">
         <v>0.16770239264019773</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21">
         <v>0.8689188074153279</v>
       </c>
-      <c r="F21" s="2">
+      <c r="F21">
         <v>-103.1860989089447</v>
       </c>
-      <c r="G21" s="2">
+      <c r="G21">
         <v>120.91433362870958</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21">
         <v>-103.1860989089447</v>
       </c>
-      <c r="I21" s="2">
+      <c r="I21">
         <v>120.91433362870958</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B22" s="2">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>10</v>
+      </c>
+      <c r="B22">
         <v>-129.72128279586477</v>
       </c>
-      <c r="C22" s="2">
+      <c r="C22">
         <v>52.856236696039531</v>
       </c>
-      <c r="D22" s="2">
+      <c r="D22">
         <v>-2.4542285055565576</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22">
         <v>2.5952149163751114E-2</v>
       </c>
-      <c r="F22" s="2">
+      <c r="F22">
         <v>-241.77149906469191</v>
       </c>
-      <c r="G22" s="2">
+      <c r="G22">
         <v>-17.67106652703761</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22">
         <v>-241.77149906469191</v>
       </c>
-      <c r="I22" s="2">
+      <c r="I22">
         <v>-17.67106652703761</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="B23" s="2">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>11</v>
+      </c>
+      <c r="B23">
         <v>-13.730266984109008</v>
       </c>
-      <c r="C23" s="2">
+      <c r="C23">
         <v>52.85623669603951</v>
       </c>
-      <c r="D23" s="2">
+      <c r="D23">
         <v>-0.25976626113333962</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23">
         <v>0.79835705149469427</v>
       </c>
-      <c r="F23" s="2">
+      <c r="F23">
         <v>-125.78048325293612</v>
       </c>
-      <c r="G23" s="2">
+      <c r="G23">
         <v>98.319949284718106</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23">
         <v>-125.78048325293612</v>
       </c>
-      <c r="I23" s="2">
+      <c r="I23">
         <v>98.319949284718106</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B24" s="3">
+    <row r="24" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B24" s="2">
         <v>21.857650642124792</v>
       </c>
-      <c r="C24" s="3">
+      <c r="C24" s="2">
         <v>52.856236696039531</v>
       </c>
-      <c r="D24" s="3">
+      <c r="D24" s="2">
         <v>0.41353020964813703</v>
       </c>
-      <c r="E24" s="3">
+      <c r="E24" s="2">
         <v>0.68470780742038273</v>
       </c>
-      <c r="F24" s="3">
+      <c r="F24" s="2">
         <v>-90.192565626702361</v>
       </c>
-      <c r="G24" s="3">
+      <c r="G24" s="2">
         <v>133.90786691095195</v>
       </c>
-      <c r="H24" s="3">
+      <c r="H24" s="2">
         <v>-90.192565626702361</v>
       </c>
-      <c r="I24" s="3">
+      <c r="I24" s="2">
         <v>133.90786691095195</v>
       </c>
     </row>
@@ -987,9 +953,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q25"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1017,29 +983,29 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="K1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="L1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="M1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1077,23 +1043,23 @@
         <v>1</v>
       </c>
       <c r="N2">
-        <f>C2*D2</f>
+        <f t="shared" ref="N2:N25" si="0">C2*D2</f>
         <v>1</v>
       </c>
       <c r="O2">
-        <f>C2*E2</f>
+        <f t="shared" ref="O2:O25" si="1">C2*E2</f>
         <v>1</v>
       </c>
       <c r="P2">
-        <f>E2*D2</f>
+        <f t="shared" ref="P2:P25" si="2">E2*D2</f>
         <v>1</v>
       </c>
       <c r="Q2">
-        <f>C2*D2*E2</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+        <f t="shared" ref="Q2:Q25" si="3">C2*D2*E2</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
@@ -1131,23 +1097,23 @@
         <v>1</v>
       </c>
       <c r="N3">
-        <f>C3*D3</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="O3">
-        <f>C3*E3</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="P3">
-        <f>E3*D3</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="Q3">
-        <f>C3*D3*E3</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>1</v>
       </c>
@@ -1185,23 +1151,23 @@
         <v>1</v>
       </c>
       <c r="N4">
-        <f>C4*D4</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="O4">
-        <f>C4*E4</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="P4">
-        <f>E4*D4</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="Q4">
-        <f>C4*D4*E4</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2</v>
       </c>
@@ -1239,23 +1205,23 @@
         <v>-1</v>
       </c>
       <c r="N5">
-        <f>C5*D5</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="O5">
-        <f>C5*E5</f>
+        <f t="shared" si="1"/>
         <v>-1</v>
       </c>
       <c r="P5">
-        <f>E5*D5</f>
+        <f t="shared" si="2"/>
         <v>-1</v>
       </c>
       <c r="Q5">
-        <f>C5*D5*E5</f>
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>2</v>
       </c>
@@ -1293,23 +1259,23 @@
         <v>-1</v>
       </c>
       <c r="N6">
-        <f>C6*D6</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="O6">
-        <f>C6*E6</f>
+        <f t="shared" si="1"/>
         <v>-1</v>
       </c>
       <c r="P6">
-        <f>E6*D6</f>
+        <f t="shared" si="2"/>
         <v>-1</v>
       </c>
       <c r="Q6">
-        <f>C6*D6*E6</f>
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>2</v>
       </c>
@@ -1347,23 +1313,23 @@
         <v>-1</v>
       </c>
       <c r="N7">
-        <f>C7*D7</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="O7">
-        <f>C7*E7</f>
+        <f t="shared" si="1"/>
         <v>-1</v>
       </c>
       <c r="P7">
-        <f>E7*D7</f>
+        <f t="shared" si="2"/>
         <v>-1</v>
       </c>
       <c r="Q7">
-        <f>C7*D7*E7</f>
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>3</v>
       </c>
@@ -1401,23 +1367,23 @@
         <v>1</v>
       </c>
       <c r="N8">
-        <f>C8*D8</f>
+        <f t="shared" si="0"/>
         <v>-1</v>
       </c>
       <c r="O8">
-        <f>C8*E8</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="P8">
-        <f>E8*D8</f>
+        <f t="shared" si="2"/>
         <v>-1</v>
       </c>
       <c r="Q8">
-        <f>C8*D8*E8</f>
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>3</v>
       </c>
@@ -1455,23 +1421,23 @@
         <v>1</v>
       </c>
       <c r="N9">
-        <f>C9*D9</f>
+        <f t="shared" si="0"/>
         <v>-1</v>
       </c>
       <c r="O9">
-        <f>C9*E9</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="P9">
-        <f>E9*D9</f>
+        <f t="shared" si="2"/>
         <v>-1</v>
       </c>
       <c r="Q9">
-        <f>C9*D9*E9</f>
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>3</v>
       </c>
@@ -1509,23 +1475,23 @@
         <v>1</v>
       </c>
       <c r="N10">
-        <f>C10*D10</f>
+        <f t="shared" si="0"/>
         <v>-1</v>
       </c>
       <c r="O10">
-        <f>C10*E10</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="P10">
-        <f>E10*D10</f>
+        <f t="shared" si="2"/>
         <v>-1</v>
       </c>
       <c r="Q10">
-        <f>C10*D10*E10</f>
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>4</v>
       </c>
@@ -1563,23 +1529,23 @@
         <v>-1</v>
       </c>
       <c r="N11">
-        <f>C11*D11</f>
+        <f t="shared" si="0"/>
         <v>-1</v>
       </c>
       <c r="O11">
-        <f>C11*E11</f>
+        <f t="shared" si="1"/>
         <v>-1</v>
       </c>
       <c r="P11">
-        <f>E11*D11</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="Q11">
-        <f>C11*D11*E11</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>4</v>
       </c>
@@ -1617,23 +1583,23 @@
         <v>-1</v>
       </c>
       <c r="N12">
-        <f>C12*D12</f>
+        <f t="shared" si="0"/>
         <v>-1</v>
       </c>
       <c r="O12">
-        <f>C12*E12</f>
+        <f t="shared" si="1"/>
         <v>-1</v>
       </c>
       <c r="P12">
-        <f>E12*D12</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="Q12">
-        <f>C12*D12*E12</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>4</v>
       </c>
@@ -1671,23 +1637,23 @@
         <v>-1</v>
       </c>
       <c r="N13">
-        <f>C13*D13</f>
+        <f t="shared" si="0"/>
         <v>-1</v>
       </c>
       <c r="O13">
-        <f>C13*E13</f>
+        <f t="shared" si="1"/>
         <v>-1</v>
       </c>
       <c r="P13">
-        <f>E13*D13</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="Q13">
-        <f>C13*D13*E13</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>5</v>
       </c>
@@ -1725,23 +1691,23 @@
         <v>1</v>
       </c>
       <c r="N14">
-        <f>C14*D14</f>
+        <f t="shared" si="0"/>
         <v>-1</v>
       </c>
       <c r="O14">
-        <f>C14*E14</f>
+        <f t="shared" si="1"/>
         <v>-1</v>
       </c>
       <c r="P14">
-        <f>E14*D14</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="Q14">
-        <f>C14*D14*E14</f>
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>5</v>
       </c>
@@ -1779,23 +1745,23 @@
         <v>1</v>
       </c>
       <c r="N15">
-        <f>C15*D15</f>
+        <f t="shared" si="0"/>
         <v>-1</v>
       </c>
       <c r="O15">
-        <f>C15*E15</f>
+        <f t="shared" si="1"/>
         <v>-1</v>
       </c>
       <c r="P15">
-        <f>E15*D15</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="Q15">
-        <f>C15*D15*E15</f>
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>5</v>
       </c>
@@ -1833,23 +1799,23 @@
         <v>1</v>
       </c>
       <c r="N16">
-        <f>C16*D16</f>
+        <f t="shared" si="0"/>
         <v>-1</v>
       </c>
       <c r="O16">
-        <f>C16*E16</f>
+        <f t="shared" si="1"/>
         <v>-1</v>
       </c>
       <c r="P16">
-        <f>E16*D16</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="Q16">
-        <f>C16*D16*E16</f>
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>6</v>
       </c>
@@ -1887,23 +1853,23 @@
         <v>-1</v>
       </c>
       <c r="N17">
-        <f>C17*D17</f>
+        <f t="shared" si="0"/>
         <v>-1</v>
       </c>
       <c r="O17">
-        <f>C17*E17</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="P17">
-        <f>E17*D17</f>
+        <f t="shared" si="2"/>
         <v>-1</v>
       </c>
       <c r="Q17">
-        <f>C17*D17*E17</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>6</v>
       </c>
@@ -1941,23 +1907,23 @@
         <v>-1</v>
       </c>
       <c r="N18">
-        <f>C18*D18</f>
+        <f t="shared" si="0"/>
         <v>-1</v>
       </c>
       <c r="O18">
-        <f>C18*E18</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="P18">
-        <f>E18*D18</f>
+        <f t="shared" si="2"/>
         <v>-1</v>
       </c>
       <c r="Q18">
-        <f>C18*D18*E18</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>6</v>
       </c>
@@ -1995,23 +1961,23 @@
         <v>-1</v>
       </c>
       <c r="N19">
-        <f>C19*D19</f>
+        <f t="shared" si="0"/>
         <v>-1</v>
       </c>
       <c r="O19">
-        <f>C19*E19</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="P19">
-        <f>E19*D19</f>
+        <f t="shared" si="2"/>
         <v>-1</v>
       </c>
       <c r="Q19">
-        <f>C19*D19*E19</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>7</v>
       </c>
@@ -2049,23 +2015,23 @@
         <v>1</v>
       </c>
       <c r="N20">
-        <f>C20*D20</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="O20">
-        <f>C20*E20</f>
+        <f t="shared" si="1"/>
         <v>-1</v>
       </c>
       <c r="P20">
-        <f>E20*D20</f>
+        <f t="shared" si="2"/>
         <v>-1</v>
       </c>
       <c r="Q20">
-        <f>C20*D20*E20</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>7</v>
       </c>
@@ -2103,23 +2069,23 @@
         <v>1</v>
       </c>
       <c r="N21">
-        <f>C21*D21</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="O21">
-        <f>C21*E21</f>
+        <f t="shared" si="1"/>
         <v>-1</v>
       </c>
       <c r="P21">
-        <f>E21*D21</f>
+        <f t="shared" si="2"/>
         <v>-1</v>
       </c>
       <c r="Q21">
-        <f>C21*D21*E21</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>7</v>
       </c>
@@ -2157,23 +2123,23 @@
         <v>1</v>
       </c>
       <c r="N22">
-        <f>C22*D22</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="O22">
-        <f>C22*E22</f>
+        <f t="shared" si="1"/>
         <v>-1</v>
       </c>
       <c r="P22">
-        <f>E22*D22</f>
+        <f t="shared" si="2"/>
         <v>-1</v>
       </c>
       <c r="Q22">
-        <f>C22*D22*E22</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>8</v>
       </c>
@@ -2211,23 +2177,23 @@
         <v>-1</v>
       </c>
       <c r="N23">
-        <f>C23*D23</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="O23">
-        <f>C23*E23</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="P23">
-        <f>E23*D23</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="Q23">
-        <f>C23*D23*E23</f>
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>8</v>
       </c>
@@ -2265,23 +2231,23 @@
         <v>-1</v>
       </c>
       <c r="N24">
-        <f>C24*D24</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="O24">
-        <f>C24*E24</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="P24">
-        <f>E24*D24</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="Q24">
-        <f>C24*D24*E24</f>
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
+        <f t="shared" si="3"/>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>8</v>
       </c>
@@ -2319,19 +2285,19 @@
         <v>-1</v>
       </c>
       <c r="N25">
-        <f>C25*D25</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="O25">
-        <f>C25*E25</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="P25">
-        <f>E25*D25</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="Q25">
-        <f>C25*D25*E25</f>
+        <f t="shared" si="3"/>
         <v>-1</v>
       </c>
     </row>

</xml_diff>